<commit_message>
Deploying to gh-pages from  @ fb0862f86dbab6133b8835a84d0e554ff8d14ceb 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/10.1.1.xlsx
+++ b/en/downloads/data-excel/10.1.1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="60" windowWidth="28800" windowHeight="12375"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -206,7 +206,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -256,6 +256,15 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -563,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="41" style="1" customWidth="1"/>
@@ -571,7 +580,7 @@
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
@@ -590,7 +599,7 @@
       <c r="J1" s="13"/>
       <c r="K1" s="13"/>
     </row>
-    <row r="2" spans="1:12" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -609,7 +618,7 @@
       <c r="J2" s="13"/>
       <c r="K2" s="13"/>
     </row>
-    <row r="3" spans="1:12" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14"/>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -622,7 +631,7 @@
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
@@ -659,8 +668,11 @@
       <c r="L4" s="18">
         <v>2023</v>
       </c>
+      <c r="M4" s="19">
+        <v>2024</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>9</v>
       </c>
@@ -697,8 +709,11 @@
       <c r="L5" s="7">
         <v>4.9000000000000004</v>
       </c>
+      <c r="M5" s="20">
+        <v>6.7</v>
+      </c>
     </row>
-    <row r="6" spans="1:12" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>8</v>
       </c>
@@ -734,6 +749,9 @@
       </c>
       <c r="L6" s="11">
         <v>4.5999999999999996</v>
+      </c>
+      <c r="M6" s="21">
+        <v>4.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>